<commit_message>
Added new RDF data schemes and visual schemes for economy-table121-123, fixed XLSX spreadsheet for economy-table123
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/economy-table123.xlsx
+++ b/sources/table_normalization/xlsx/economy-table123.xlsx
@@ -91,8 +91,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="2">
-    <numFmt numFmtId="168" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="169" formatCode="_-\$* #,##0.00_ ;_-\$* \-#,##0.00\ ;_-\$* &quot;-&quot;??_ ;_-@_ "/>
+    <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="_-\$* #,##0.00_ ;_-\$* \-#,##0.00\ ;_-\$* &quot;-&quot;??_ ;_-@_ "/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -116,7 +116,7 @@
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -126,12 +126,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00B0F0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -202,12 +196,9 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="17" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -216,8 +207,11 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="168" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="169" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -227,14 +221,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="168" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -726,52 +712,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="A1" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="10" t="s">
+      <c r="A1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2">
+      <c r="D1" s="1">
         <v>41640</v>
       </c>
-      <c r="E1" s="2">
+      <c r="E1" s="1">
         <v>41671</v>
       </c>
-      <c r="F1" s="2">
+      <c r="F1" s="1">
         <v>41699</v>
       </c>
-      <c r="G1" s="2">
+      <c r="G1" s="1">
         <v>41730</v>
       </c>
-      <c r="H1" s="2">
+      <c r="H1" s="1">
         <v>41760</v>
       </c>
-      <c r="I1" s="2">
+      <c r="I1" s="1">
         <v>41791</v>
       </c>
-      <c r="J1" s="2">
+      <c r="J1" s="1">
         <v>41821</v>
       </c>
-      <c r="K1" s="2">
+      <c r="K1" s="1">
         <v>41852</v>
       </c>
-      <c r="L1" s="2">
+      <c r="L1" s="1">
         <v>41883</v>
       </c>
-      <c r="M1" s="2">
+      <c r="M1" s="1">
         <v>41913</v>
       </c>
-      <c r="N1" s="2">
+      <c r="N1" s="1">
         <v>41944</v>
       </c>
-      <c r="O1" s="2">
+      <c r="O1" s="1">
         <v>41974</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" s="6" t="s">
         <v>3</v>
       </c>
     </row>
@@ -779,739 +765,739 @@
       <c r="A2" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="5">
+      <c r="C2" s="3"/>
+      <c r="D2" s="4">
         <v>40</v>
       </c>
-      <c r="E2" s="5">
+      <c r="E2" s="4">
         <v>40</v>
       </c>
-      <c r="F2" s="5">
+      <c r="F2" s="4">
         <v>40</v>
       </c>
-      <c r="G2" s="5">
+      <c r="G2" s="4">
         <v>40</v>
       </c>
-      <c r="H2" s="5">
+      <c r="H2" s="4">
         <v>40</v>
       </c>
-      <c r="I2" s="5">
-        <v>50</v>
-      </c>
-      <c r="J2" s="5">
-        <v>50</v>
-      </c>
-      <c r="K2" s="5">
-        <v>50</v>
-      </c>
-      <c r="L2" s="5">
+      <c r="I2" s="4">
+        <v>50</v>
+      </c>
+      <c r="J2" s="4">
+        <v>50</v>
+      </c>
+      <c r="K2" s="4">
+        <v>50</v>
+      </c>
+      <c r="L2" s="4">
         <v>40</v>
       </c>
-      <c r="M2" s="5">
-        <v>50</v>
-      </c>
-      <c r="N2" s="5">
-        <v>50</v>
-      </c>
-      <c r="O2" s="5">
+      <c r="M2" s="4">
+        <v>50</v>
+      </c>
+      <c r="N2" s="4">
+        <v>50</v>
+      </c>
+      <c r="O2" s="4">
         <v>40</v>
       </c>
-      <c r="P2" s="5">
+      <c r="P2" s="4">
         <f t="shared" ref="P2:P8" si="0">SUM(D2:O2)</f>
         <v>530</v>
       </c>
     </row>
     <row r="3" spans="1:16">
       <c r="A3" s="8"/>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="5">
-        <v>50</v>
-      </c>
-      <c r="E3" s="5">
-        <v>50</v>
-      </c>
-      <c r="F3" s="5">
-        <v>50</v>
-      </c>
-      <c r="G3" s="5">
-        <v>50</v>
-      </c>
-      <c r="H3" s="5">
-        <v>50</v>
-      </c>
-      <c r="I3" s="5">
+      <c r="C3" s="3"/>
+      <c r="D3" s="4">
+        <v>50</v>
+      </c>
+      <c r="E3" s="4">
+        <v>50</v>
+      </c>
+      <c r="F3" s="4">
+        <v>50</v>
+      </c>
+      <c r="G3" s="4">
+        <v>50</v>
+      </c>
+      <c r="H3" s="4">
+        <v>50</v>
+      </c>
+      <c r="I3" s="4">
         <v>60</v>
       </c>
-      <c r="J3" s="5">
+      <c r="J3" s="4">
         <v>60</v>
       </c>
-      <c r="K3" s="5">
+      <c r="K3" s="4">
         <v>60</v>
       </c>
-      <c r="L3" s="5">
-        <v>50</v>
-      </c>
-      <c r="M3" s="5">
+      <c r="L3" s="4">
+        <v>50</v>
+      </c>
+      <c r="M3" s="4">
         <v>60</v>
       </c>
-      <c r="N3" s="5">
+      <c r="N3" s="4">
         <v>60</v>
       </c>
-      <c r="O3" s="5">
-        <v>50</v>
-      </c>
-      <c r="P3" s="5">
+      <c r="O3" s="4">
+        <v>50</v>
+      </c>
+      <c r="P3" s="4">
         <f t="shared" si="0"/>
         <v>650</v>
       </c>
     </row>
     <row r="4" spans="1:16">
       <c r="A4" s="9"/>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="5">
+      <c r="C4" s="3"/>
+      <c r="D4" s="4">
         <f t="shared" ref="D4:O4" si="1">D2+D3</f>
         <v>90</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="4">
         <f t="shared" si="1"/>
         <v>90</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="4">
         <f t="shared" si="1"/>
         <v>90</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="4">
         <f t="shared" si="1"/>
         <v>90</v>
       </c>
-      <c r="H4" s="5">
+      <c r="H4" s="4">
         <f t="shared" si="1"/>
         <v>90</v>
       </c>
-      <c r="I4" s="5">
+      <c r="I4" s="4">
         <f t="shared" si="1"/>
         <v>110</v>
       </c>
-      <c r="J4" s="5">
+      <c r="J4" s="4">
         <f t="shared" si="1"/>
         <v>110</v>
       </c>
-      <c r="K4" s="5">
+      <c r="K4" s="4">
         <f t="shared" si="1"/>
         <v>110</v>
       </c>
-      <c r="L4" s="5">
+      <c r="L4" s="4">
         <f t="shared" si="1"/>
         <v>90</v>
       </c>
-      <c r="M4" s="5">
+      <c r="M4" s="4">
         <f t="shared" si="1"/>
         <v>110</v>
       </c>
-      <c r="N4" s="5">
+      <c r="N4" s="4">
         <f t="shared" si="1"/>
         <v>110</v>
       </c>
-      <c r="O4" s="5">
+      <c r="O4" s="4">
         <f t="shared" si="1"/>
         <v>90</v>
       </c>
-      <c r="P4" s="5">
+      <c r="P4" s="4">
         <f t="shared" si="0"/>
         <v>1180</v>
       </c>
     </row>
     <row r="5" spans="1:16">
-      <c r="A5" s="11"/>
-      <c r="B5" s="11"/>
-      <c r="C5" s="12"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="13"/>
-      <c r="F5" s="13"/>
-      <c r="G5" s="13"/>
-      <c r="H5" s="13"/>
-      <c r="I5" s="13"/>
-      <c r="J5" s="13"/>
-      <c r="K5" s="13"/>
-      <c r="L5" s="13"/>
-      <c r="M5" s="13"/>
-      <c r="N5" s="13"/>
-      <c r="O5" s="13"/>
-      <c r="P5" s="13"/>
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="4"/>
+      <c r="K5" s="4"/>
+      <c r="L5" s="4"/>
+      <c r="M5" s="4"/>
+      <c r="N5" s="4"/>
+      <c r="O5" s="4"/>
+      <c r="P5" s="4"/>
     </row>
     <row r="6" spans="1:16">
       <c r="A6" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="5">
-        <v>10</v>
-      </c>
-      <c r="E6" s="5">
-        <v>10</v>
-      </c>
-      <c r="F6" s="5">
-        <v>10</v>
-      </c>
-      <c r="G6" s="5">
-        <v>10</v>
-      </c>
-      <c r="H6" s="5">
-        <v>10</v>
-      </c>
-      <c r="I6" s="5">
-        <v>20</v>
-      </c>
-      <c r="J6" s="5">
-        <v>20</v>
-      </c>
-      <c r="K6" s="5">
-        <v>20</v>
-      </c>
-      <c r="L6" s="5">
-        <v>10</v>
-      </c>
-      <c r="M6" s="5">
-        <v>20</v>
-      </c>
-      <c r="N6" s="5">
-        <v>20</v>
-      </c>
-      <c r="O6" s="5">
-        <v>10</v>
-      </c>
-      <c r="P6" s="5">
+      <c r="C6" s="3"/>
+      <c r="D6" s="4">
+        <v>10</v>
+      </c>
+      <c r="E6" s="4">
+        <v>10</v>
+      </c>
+      <c r="F6" s="4">
+        <v>10</v>
+      </c>
+      <c r="G6" s="4">
+        <v>10</v>
+      </c>
+      <c r="H6" s="4">
+        <v>10</v>
+      </c>
+      <c r="I6" s="4">
+        <v>20</v>
+      </c>
+      <c r="J6" s="4">
+        <v>20</v>
+      </c>
+      <c r="K6" s="4">
+        <v>20</v>
+      </c>
+      <c r="L6" s="4">
+        <v>10</v>
+      </c>
+      <c r="M6" s="4">
+        <v>20</v>
+      </c>
+      <c r="N6" s="4">
+        <v>20</v>
+      </c>
+      <c r="O6" s="4">
+        <v>10</v>
+      </c>
+      <c r="P6" s="4">
         <f t="shared" si="0"/>
         <v>170</v>
       </c>
     </row>
     <row r="7" spans="1:16">
       <c r="A7" s="8"/>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="5">
-        <v>10</v>
-      </c>
-      <c r="E7" s="5">
-        <v>10</v>
-      </c>
-      <c r="F7" s="5">
-        <v>10</v>
-      </c>
-      <c r="G7" s="5">
-        <v>10</v>
-      </c>
-      <c r="H7" s="5">
-        <v>10</v>
-      </c>
-      <c r="I7" s="5">
+      <c r="C7" s="3"/>
+      <c r="D7" s="4">
+        <v>10</v>
+      </c>
+      <c r="E7" s="4">
+        <v>10</v>
+      </c>
+      <c r="F7" s="4">
+        <v>10</v>
+      </c>
+      <c r="G7" s="4">
+        <v>10</v>
+      </c>
+      <c r="H7" s="4">
+        <v>10</v>
+      </c>
+      <c r="I7" s="4">
         <v>40</v>
       </c>
-      <c r="J7" s="5">
+      <c r="J7" s="4">
         <v>40</v>
       </c>
-      <c r="K7" s="5">
+      <c r="K7" s="4">
         <v>40</v>
       </c>
-      <c r="L7" s="5">
-        <v>10</v>
-      </c>
-      <c r="M7" s="5">
+      <c r="L7" s="4">
+        <v>10</v>
+      </c>
+      <c r="M7" s="4">
         <v>40</v>
       </c>
-      <c r="N7" s="5">
+      <c r="N7" s="4">
         <v>40</v>
       </c>
-      <c r="O7" s="5">
-        <v>10</v>
-      </c>
-      <c r="P7" s="5">
+      <c r="O7" s="4">
+        <v>10</v>
+      </c>
+      <c r="P7" s="4">
         <f t="shared" si="0"/>
         <v>270</v>
       </c>
     </row>
     <row r="8" spans="1:16">
       <c r="A8" s="9"/>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="4"/>
-      <c r="D8" s="5">
+      <c r="C8" s="3"/>
+      <c r="D8" s="4">
         <f t="shared" ref="D8:O8" si="2">D6+D7</f>
         <v>20</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="4">
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="F8" s="5">
+      <c r="F8" s="4">
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="G8" s="5">
+      <c r="G8" s="4">
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="H8" s="5">
+      <c r="H8" s="4">
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="I8" s="5">
+      <c r="I8" s="4">
         <f t="shared" si="2"/>
         <v>60</v>
       </c>
-      <c r="J8" s="5">
+      <c r="J8" s="4">
         <f t="shared" si="2"/>
         <v>60</v>
       </c>
-      <c r="K8" s="5">
+      <c r="K8" s="4">
         <f t="shared" si="2"/>
         <v>60</v>
       </c>
-      <c r="L8" s="5">
+      <c r="L8" s="4">
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="M8" s="5">
+      <c r="M8" s="4">
         <f t="shared" si="2"/>
         <v>60</v>
       </c>
-      <c r="N8" s="5">
+      <c r="N8" s="4">
         <f t="shared" si="2"/>
         <v>60</v>
       </c>
-      <c r="O8" s="5">
+      <c r="O8" s="4">
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="P8" s="5">
+      <c r="P8" s="4">
         <f t="shared" si="0"/>
         <v>440</v>
       </c>
     </row>
     <row r="9" spans="1:16">
-      <c r="A9" s="11"/>
-      <c r="B9" s="11"/>
-      <c r="C9" s="12"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="13"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="13"/>
-      <c r="H9" s="13"/>
-      <c r="I9" s="13"/>
-      <c r="J9" s="13"/>
-      <c r="K9" s="13"/>
-      <c r="L9" s="13"/>
-      <c r="M9" s="13"/>
-      <c r="N9" s="13"/>
-      <c r="O9" s="13"/>
-      <c r="P9" s="13"/>
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="4"/>
+      <c r="H9" s="4"/>
+      <c r="I9" s="4"/>
+      <c r="J9" s="4"/>
+      <c r="K9" s="4"/>
+      <c r="L9" s="4"/>
+      <c r="M9" s="4"/>
+      <c r="N9" s="4"/>
+      <c r="O9" s="4"/>
+      <c r="P9" s="4"/>
     </row>
     <row r="10" spans="1:16">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C10" s="4"/>
-      <c r="D10" s="5">
+      <c r="B10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10" s="3"/>
+      <c r="D10" s="4">
         <f t="shared" ref="D10:O10" si="3">D4-D8</f>
         <v>70</v>
       </c>
-      <c r="E10" s="5">
+      <c r="E10" s="4">
         <f t="shared" si="3"/>
         <v>70</v>
       </c>
-      <c r="F10" s="5">
+      <c r="F10" s="4">
         <f t="shared" si="3"/>
         <v>70</v>
       </c>
-      <c r="G10" s="5">
+      <c r="G10" s="4">
         <f t="shared" si="3"/>
         <v>70</v>
       </c>
-      <c r="H10" s="5">
+      <c r="H10" s="4">
         <f t="shared" si="3"/>
         <v>70</v>
       </c>
-      <c r="I10" s="5">
+      <c r="I10" s="4">
         <f t="shared" si="3"/>
         <v>50</v>
       </c>
-      <c r="J10" s="5">
+      <c r="J10" s="4">
         <f t="shared" si="3"/>
         <v>50</v>
       </c>
-      <c r="K10" s="5">
+      <c r="K10" s="4">
         <f t="shared" si="3"/>
         <v>50</v>
       </c>
-      <c r="L10" s="5">
+      <c r="L10" s="4">
         <f t="shared" si="3"/>
         <v>70</v>
       </c>
-      <c r="M10" s="5">
+      <c r="M10" s="4">
         <f t="shared" si="3"/>
         <v>50</v>
       </c>
-      <c r="N10" s="5">
+      <c r="N10" s="4">
         <f t="shared" si="3"/>
         <v>50</v>
       </c>
-      <c r="O10" s="5">
+      <c r="O10" s="4">
         <f t="shared" si="3"/>
         <v>70</v>
       </c>
-      <c r="P10" s="5">
+      <c r="P10" s="4">
         <f>SUM(D10:O10)</f>
         <v>740</v>
       </c>
     </row>
     <row r="11" spans="1:16">
-      <c r="A11" s="11"/>
-      <c r="B11" s="11"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13"/>
-      <c r="G11" s="13"/>
-      <c r="H11" s="13"/>
-      <c r="I11" s="13"/>
-      <c r="J11" s="13"/>
-      <c r="K11" s="13"/>
-      <c r="L11" s="13"/>
-      <c r="M11" s="13"/>
-      <c r="N11" s="13"/>
-      <c r="O11" s="13"/>
-      <c r="P11" s="13"/>
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="4"/>
+      <c r="H11" s="4"/>
+      <c r="I11" s="4"/>
+      <c r="J11" s="4"/>
+      <c r="K11" s="4"/>
+      <c r="L11" s="4"/>
+      <c r="M11" s="4"/>
+      <c r="N11" s="4"/>
+      <c r="O11" s="4"/>
+      <c r="P11" s="4"/>
     </row>
     <row r="12" spans="1:16">
       <c r="A12" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="4"/>
-      <c r="D12" s="5">
-        <v>0</v>
-      </c>
-      <c r="E12" s="5">
-        <v>0</v>
-      </c>
-      <c r="F12" s="5">
-        <v>0</v>
-      </c>
-      <c r="G12" s="5">
-        <v>0</v>
-      </c>
-      <c r="H12" s="5">
-        <v>0</v>
-      </c>
-      <c r="I12" s="5">
-        <v>0</v>
-      </c>
-      <c r="J12" s="5">
-        <v>0</v>
-      </c>
-      <c r="K12" s="5">
-        <v>0</v>
-      </c>
-      <c r="L12" s="5">
-        <v>0</v>
-      </c>
-      <c r="M12" s="5">
-        <v>0</v>
-      </c>
-      <c r="N12" s="5">
-        <v>0</v>
-      </c>
-      <c r="O12" s="5">
-        <v>0</v>
-      </c>
-      <c r="P12" s="5">
+      <c r="C12" s="3"/>
+      <c r="D12" s="4">
+        <v>0</v>
+      </c>
+      <c r="E12" s="4">
+        <v>0</v>
+      </c>
+      <c r="F12" s="4">
+        <v>0</v>
+      </c>
+      <c r="G12" s="4">
+        <v>0</v>
+      </c>
+      <c r="H12" s="4">
+        <v>0</v>
+      </c>
+      <c r="I12" s="4">
+        <v>0</v>
+      </c>
+      <c r="J12" s="4">
+        <v>0</v>
+      </c>
+      <c r="K12" s="4">
+        <v>0</v>
+      </c>
+      <c r="L12" s="4">
+        <v>0</v>
+      </c>
+      <c r="M12" s="4">
+        <v>0</v>
+      </c>
+      <c r="N12" s="4">
+        <v>0</v>
+      </c>
+      <c r="O12" s="4">
+        <v>0</v>
+      </c>
+      <c r="P12" s="4">
         <f>SUM(D12:O12)</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:16">
       <c r="A13" s="8"/>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="4"/>
-      <c r="D13" s="5">
-        <v>0</v>
-      </c>
-      <c r="E13" s="5">
-        <v>0</v>
-      </c>
-      <c r="F13" s="5">
-        <v>0</v>
-      </c>
-      <c r="G13" s="5">
-        <v>0</v>
-      </c>
-      <c r="H13" s="5">
-        <v>0</v>
-      </c>
-      <c r="I13" s="5">
-        <v>0</v>
-      </c>
-      <c r="J13" s="5">
-        <v>0</v>
-      </c>
-      <c r="K13" s="5">
-        <v>0</v>
-      </c>
-      <c r="L13" s="5">
-        <v>0</v>
-      </c>
-      <c r="M13" s="5">
-        <v>0</v>
-      </c>
-      <c r="N13" s="5">
-        <v>0</v>
-      </c>
-      <c r="O13" s="5">
-        <v>0</v>
-      </c>
-      <c r="P13" s="5">
+      <c r="C13" s="3"/>
+      <c r="D13" s="4">
+        <v>0</v>
+      </c>
+      <c r="E13" s="4">
+        <v>0</v>
+      </c>
+      <c r="F13" s="4">
+        <v>0</v>
+      </c>
+      <c r="G13" s="4">
+        <v>0</v>
+      </c>
+      <c r="H13" s="4">
+        <v>0</v>
+      </c>
+      <c r="I13" s="4">
+        <v>0</v>
+      </c>
+      <c r="J13" s="4">
+        <v>0</v>
+      </c>
+      <c r="K13" s="4">
+        <v>0</v>
+      </c>
+      <c r="L13" s="4">
+        <v>0</v>
+      </c>
+      <c r="M13" s="4">
+        <v>0</v>
+      </c>
+      <c r="N13" s="4">
+        <v>0</v>
+      </c>
+      <c r="O13" s="4">
+        <v>0</v>
+      </c>
+      <c r="P13" s="4">
         <f>SUM(D13:O13)</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:16">
       <c r="A14" s="8"/>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="4"/>
-      <c r="D14" s="5">
-        <v>20</v>
-      </c>
-      <c r="E14" s="5">
-        <v>20</v>
-      </c>
-      <c r="F14" s="5">
-        <v>20</v>
-      </c>
-      <c r="G14" s="5">
-        <v>20</v>
-      </c>
-      <c r="H14" s="5">
-        <v>20</v>
-      </c>
-      <c r="I14" s="5">
-        <v>10</v>
-      </c>
-      <c r="J14" s="5">
-        <v>10</v>
-      </c>
-      <c r="K14" s="5">
-        <v>10</v>
-      </c>
-      <c r="L14" s="5">
-        <v>20</v>
-      </c>
-      <c r="M14" s="5">
-        <v>10</v>
-      </c>
-      <c r="N14" s="5">
-        <v>10</v>
-      </c>
-      <c r="O14" s="5">
-        <v>20</v>
-      </c>
-      <c r="P14" s="5">
+      <c r="C14" s="3"/>
+      <c r="D14" s="4">
+        <v>20</v>
+      </c>
+      <c r="E14" s="4">
+        <v>20</v>
+      </c>
+      <c r="F14" s="4">
+        <v>20</v>
+      </c>
+      <c r="G14" s="4">
+        <v>20</v>
+      </c>
+      <c r="H14" s="4">
+        <v>20</v>
+      </c>
+      <c r="I14" s="4">
+        <v>10</v>
+      </c>
+      <c r="J14" s="4">
+        <v>10</v>
+      </c>
+      <c r="K14" s="4">
+        <v>10</v>
+      </c>
+      <c r="L14" s="4">
+        <v>20</v>
+      </c>
+      <c r="M14" s="4">
+        <v>10</v>
+      </c>
+      <c r="N14" s="4">
+        <v>10</v>
+      </c>
+      <c r="O14" s="4">
+        <v>20</v>
+      </c>
+      <c r="P14" s="4">
         <f>SUM(D14:O14)</f>
         <v>190</v>
       </c>
     </row>
     <row r="15" spans="1:16">
       <c r="A15" s="8"/>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="4"/>
-      <c r="D15" s="5">
+      <c r="C15" s="3"/>
+      <c r="D15" s="4">
         <v>30</v>
       </c>
-      <c r="E15" s="5">
+      <c r="E15" s="4">
         <v>30</v>
       </c>
-      <c r="F15" s="5">
+      <c r="F15" s="4">
         <v>30</v>
       </c>
-      <c r="G15" s="5">
+      <c r="G15" s="4">
         <v>30</v>
       </c>
-      <c r="H15" s="5">
+      <c r="H15" s="4">
         <v>30</v>
       </c>
-      <c r="I15" s="5">
-        <v>20</v>
-      </c>
-      <c r="J15" s="5">
-        <v>20</v>
-      </c>
-      <c r="K15" s="5">
-        <v>20</v>
-      </c>
-      <c r="L15" s="5">
+      <c r="I15" s="4">
+        <v>20</v>
+      </c>
+      <c r="J15" s="4">
+        <v>20</v>
+      </c>
+      <c r="K15" s="4">
+        <v>20</v>
+      </c>
+      <c r="L15" s="4">
         <v>30</v>
       </c>
-      <c r="M15" s="5">
-        <v>20</v>
-      </c>
-      <c r="N15" s="5">
-        <v>20</v>
-      </c>
-      <c r="O15" s="5">
+      <c r="M15" s="4">
+        <v>20</v>
+      </c>
+      <c r="N15" s="4">
+        <v>20</v>
+      </c>
+      <c r="O15" s="4">
         <v>30</v>
       </c>
-      <c r="P15" s="5">
+      <c r="P15" s="4">
         <f>SUM(D15:O15)</f>
         <v>310</v>
       </c>
     </row>
     <row r="16" spans="1:16">
       <c r="A16" s="9"/>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C16" s="4"/>
-      <c r="D16" s="5">
-        <v>10</v>
-      </c>
-      <c r="E16" s="5">
-        <v>10</v>
-      </c>
-      <c r="F16" s="5">
-        <v>10</v>
-      </c>
-      <c r="G16" s="5">
-        <v>10</v>
-      </c>
-      <c r="H16" s="5">
-        <v>10</v>
-      </c>
-      <c r="I16" s="5">
+      <c r="C16" s="3"/>
+      <c r="D16" s="4">
+        <v>10</v>
+      </c>
+      <c r="E16" s="4">
+        <v>10</v>
+      </c>
+      <c r="F16" s="4">
+        <v>10</v>
+      </c>
+      <c r="G16" s="4">
+        <v>10</v>
+      </c>
+      <c r="H16" s="4">
+        <v>10</v>
+      </c>
+      <c r="I16" s="4">
         <v>54</v>
       </c>
-      <c r="J16" s="5">
+      <c r="J16" s="4">
         <v>54</v>
       </c>
-      <c r="K16" s="5">
+      <c r="K16" s="4">
         <v>54</v>
       </c>
-      <c r="L16" s="5">
-        <v>10</v>
-      </c>
-      <c r="M16" s="5">
+      <c r="L16" s="4">
+        <v>10</v>
+      </c>
+      <c r="M16" s="4">
         <v>54</v>
       </c>
-      <c r="N16" s="5">
+      <c r="N16" s="4">
         <v>54</v>
       </c>
-      <c r="O16" s="5">
-        <v>10</v>
-      </c>
-      <c r="P16" s="5">
+      <c r="O16" s="4">
+        <v>10</v>
+      </c>
+      <c r="P16" s="4">
         <f>SUM(D16:O16)</f>
         <v>340</v>
       </c>
     </row>
     <row r="17" spans="1:16">
-      <c r="A17" s="11"/>
-      <c r="B17" s="11"/>
-      <c r="C17" s="12"/>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="13"/>
-      <c r="G17" s="13"/>
-      <c r="H17" s="13"/>
-      <c r="I17" s="13"/>
-      <c r="J17" s="13"/>
-      <c r="K17" s="13"/>
-      <c r="L17" s="13"/>
-      <c r="M17" s="13"/>
-      <c r="N17" s="13"/>
-      <c r="O17" s="13"/>
-      <c r="P17" s="13"/>
+      <c r="A17" s="2"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="4"/>
+      <c r="G17" s="4"/>
+      <c r="H17" s="4"/>
+      <c r="I17" s="4"/>
+      <c r="J17" s="4"/>
+      <c r="K17" s="4"/>
+      <c r="L17" s="4"/>
+      <c r="M17" s="4"/>
+      <c r="N17" s="4"/>
+      <c r="O17" s="4"/>
+      <c r="P17" s="4"/>
     </row>
     <row r="18" spans="1:16">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C18" s="4"/>
-      <c r="D18" s="5">
+      <c r="C18" s="3"/>
+      <c r="D18" s="4">
         <f t="shared" ref="D18:O18" si="4">D10-D14-D12-D13-D15-D16</f>
         <v>10</v>
       </c>
-      <c r="E18" s="5">
+      <c r="E18" s="4">
         <f t="shared" si="4"/>
         <v>10</v>
       </c>
-      <c r="F18" s="5">
+      <c r="F18" s="4">
         <f t="shared" si="4"/>
         <v>10</v>
       </c>
-      <c r="G18" s="5">
+      <c r="G18" s="4">
         <f t="shared" si="4"/>
         <v>10</v>
       </c>
-      <c r="H18" s="5">
+      <c r="H18" s="4">
         <f t="shared" si="4"/>
         <v>10</v>
       </c>
-      <c r="I18" s="6">
+      <c r="I18" s="5">
         <f>I10-I14-I12-I13-I15-I16</f>
         <v>-34</v>
       </c>
-      <c r="J18" s="6">
+      <c r="J18" s="5">
         <f t="shared" si="4"/>
         <v>-34</v>
       </c>
-      <c r="K18" s="6">
+      <c r="K18" s="5">
         <f t="shared" si="4"/>
         <v>-34</v>
       </c>
-      <c r="L18" s="6">
+      <c r="L18" s="5">
         <f t="shared" si="4"/>
         <v>10</v>
       </c>
-      <c r="M18" s="6">
+      <c r="M18" s="5">
         <f t="shared" si="4"/>
         <v>-34</v>
       </c>
-      <c r="N18" s="6">
+      <c r="N18" s="5">
         <f t="shared" si="4"/>
         <v>-34</v>
       </c>
-      <c r="O18" s="6">
+      <c r="O18" s="5">
         <f t="shared" si="4"/>
         <v>10</v>
       </c>
-      <c r="P18" s="6">
+      <c r="P18" s="5">
         <f>SUM(D18:O18)</f>
         <v>-100</v>
       </c>

</xml_diff>